<commit_message>
fix: prefer the survey country's alias when matching columns
Spain headers were matching another country's variable id, so core columns and Spanish answers were assigned to the wrong variables. Trailing answer tags are only ID plus digits, so [COUNTRY] and codes such as (ES) stay.
</commit_message>
<xml_diff>
--- a/data/country_maps/spain_review.xlsx
+++ b/data/country_maps/spain_review.xlsx
@@ -2128,7 +2128,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>livesp1</t>
+          <t>smharm6</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2868,7 +2868,11 @@
           <t>Cooperation. Over the past six months... | Never true | Sometimes true | Often true | Prefer not to answer | You blame others for your own mistakes. | You are irritable and get angry. | You lose your temper. | You are defiant or uncooperative. | You argue or talk back to adults. | You are resentful or spiteful.</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>bcfpi_coop1</t>
+        </is>
+      </c>
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
       <c r="J56" s="5" t="inlineStr"/>
@@ -2906,7 +2910,11 @@
           <t>Managing anxiety. During the past six months... | Never true | Sometimes true | Often true | Prefer not to answer | You feel anxious or nervous about things in general. | You avoid or delay tasks due to anxiety. | You worry about being better at what you do. | You worry about your past behavior. | You worry about doing something wrong. | You worry about things in the future. | You are afraid of making mistakes.</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>bcfpi_ma1</t>
+        </is>
+      </c>
       <c r="H57" s="5" t="inlineStr"/>
       <c r="I57" s="5" t="inlineStr"/>
       <c r="J57" s="5" t="inlineStr"/>
@@ -3190,11 +3198,7 @@
           <t>School: My teachers care about me.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>bcfpi_coop1</t>
-        </is>
-      </c>
+      <c r="G63" s="2" t="n"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
           <t>Please select the response that best reflects how you have felt or behaved over the past six months. You...</t>
@@ -4310,11 +4314,7 @@
           <t>School: We learn many interesting things in school.</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
-        <is>
-          <t>bcfpi_ma1</t>
-        </is>
-      </c>
+      <c r="G93" s="2" t="n"/>
       <c r="H93" s="2" t="inlineStr">
         <is>
           <t>Please select the response that best reflects how you have felt or behaved over the past six months. You...</t>
@@ -5970,7 +5970,11 @@
           <t>Emotion regulation. During the past six months... | Never true | Sometimes true | Often true | Prefer not to answer | You have trouble controlling your emotions. | You find it very difficult to calm down when you get angry. | You feel like your emotions overwhelm you and you can't do anything about it. | You try hard not to think about your feelings. | You believe it is better to control your emotions and not think about them. | You keep your feelings to yourself.</t>
         </is>
       </c>
-      <c r="G135" s="5" t="inlineStr"/>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>bcfpi_af1</t>
+        </is>
+      </c>
       <c r="H135" s="5" t="inlineStr"/>
       <c r="I135" s="5" t="inlineStr"/>
       <c r="J135" s="5" t="inlineStr"/>
@@ -6254,11 +6258,7 @@
           <t>Relationship with parents Please indicate how often you feel this way in your family.: My parents hurt my feelings.</t>
         </is>
       </c>
-      <c r="G141" s="2" t="inlineStr">
-        <is>
-          <t>bcfpi_af1</t>
-        </is>
-      </c>
+      <c r="G141" s="2" t="n"/>
       <c r="H141" s="2" t="inlineStr">
         <is>
           <t>Please select the response that best reflects how you have felt or behaved over the past six months. You...</t>
@@ -7334,7 +7334,11 @@
           <t>Relationship with parents/guardians During your life up to now... | Always | Most of the time | Sometimes | Rarely | Never | Prefer not to answer | Did your parents / guardians understand your problems and concerns? | Did your parents / guardians really know what you did in your free time when you were not at school or work?</t>
         </is>
       </c>
-      <c r="G169" s="5" t="inlineStr"/>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>rpginsfy1</t>
+        </is>
+      </c>
       <c r="H169" s="5" t="inlineStr"/>
       <c r="I169" s="5" t="inlineStr"/>
       <c r="J169" s="5" t="inlineStr"/>
@@ -8008,7 +8012,7 @@
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>dlup1</t>
+          <t>rpginsfy2</t>
         </is>
       </c>
       <c r="H183" s="3" t="inlineStr">
@@ -8064,7 +8068,11 @@
           <t>During your life up to now... | Yes | No | Prefer not to answer | Did you live with any family member who had problems with alcohol or was an alcoholic, or who abused illegal or prescription drugs? | Did you live with any family member who was depressed, had a mental illness, or exhibited suicidal behavior? | Did you live with any family member who had been in jail or prison? | Did your parents ever separate or divorce? | Did your mother, father, or guardian pass away?</t>
         </is>
       </c>
-      <c r="G184" s="5" t="inlineStr"/>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>dlup1</t>
+        </is>
+      </c>
       <c r="H184" s="5" t="inlineStr"/>
       <c r="I184" s="5" t="inlineStr"/>
       <c r="J184" s="5" t="inlineStr"/>
@@ -9384,7 +9392,11 @@
           <t>To what extent do the following statements apply to you? | Not at all | A little | Somewhat | Quite a bit | A lot | Prefer not to answer | I have people I look up to. | Getting an education is important to me. | My parents / guardians know a lot about me. | I try to finish what I start. | I solve problems without harming myself or others (without resorting to drugs or violence). | I know where to go in my community to get help. | I feel like I belong at my school. | My family supports me in difficult times. | My friends support me in difficult times. | I am treated fairly in my community. | I have opportunities to develop skills that will be useful to me later on. | I enjoy my cultural and family traditions.</t>
         </is>
       </c>
-      <c r="G210" s="5" t="inlineStr"/>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>cyrm01</t>
+        </is>
+      </c>
       <c r="H210" s="5" t="inlineStr"/>
       <c r="I210" s="5" t="inlineStr"/>
       <c r="J210" s="5" t="inlineStr"/>
@@ -9568,11 +9580,7 @@
           <t>Relationship with friends To what extent do the following statements apply to you?: I have many friends.</t>
         </is>
       </c>
-      <c r="G214" s="2" t="inlineStr">
-        <is>
-          <t>cyrm01</t>
-        </is>
-      </c>
+      <c r="G214" s="2" t="n"/>
       <c r="H214" s="2" t="inlineStr">
         <is>
           <t>To what extent do the following statements apply to you?</t>
@@ -11458,7 +11466,11 @@
           <t>For each of the following areas of your life, indicate how often using your phone, computer, or video game console has a negative effect: | Almost always | Often | Sometimes | Rarely | Never | Prefer not to respond | Sleep. | Schoolwork. | Self-esteem / Mental health. | Relationships with friends. | Relationships with family.</t>
         </is>
       </c>
-      <c r="G251" s="5" t="inlineStr"/>
+      <c r="G251" s="5" t="inlineStr">
+        <is>
+          <t>smharm1</t>
+        </is>
+      </c>
       <c r="H251" s="5" t="inlineStr"/>
       <c r="I251" s="5" t="inlineStr"/>
       <c r="J251" s="5" t="inlineStr"/>
@@ -11492,11 +11504,7 @@
           <t>Select the option that you consider most appropriate for your situation: : I sleep less because I am using my mobile phone.</t>
         </is>
       </c>
-      <c r="G252" s="2" t="inlineStr">
-        <is>
-          <t>smharm1</t>
-        </is>
-      </c>
+      <c r="G252" s="2" t="n"/>
       <c r="H252" s="2" t="inlineStr">
         <is>
           <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>

</xml_diff>